<commit_message>
Polish sequencing workbooks; enrich from June QPRs and QPR-call decisions
Cell language made client-ready (no analyst margin notes; 'validate
w/ SPOC' removed); activities link to the business priority they
enable where warranted. New data-centre/infrastructure overlay input
row per the QPR core-team call. Integrated personas moved from a
column to inline bracket tags. Target stacks updated: disputes (WDP
north star, DMS interim, Merlin/VAP disputes demise Y1-3), payment
optimization (Revenue Boost single orchestration API; RTR+Prime
routing microservice), federated API-2.0 build model. SMB geo
priorities, constraints and milestones enriched from the June 2026
QPR regional updates (UK&I, Poland, Greece, Spain, Erste JV, Asia).

https://claude.ai/code/session_011p8iTtbymDUbCg8RtXLgqJ
</commit_message>
<xml_diff>
--- a/TAM2.0_Sequencing_Prework_Enterprise_v0.1.xlsx
+++ b/TAM2.0_Sequencing_Prework_Enterprise_v0.1.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,10 @@
     <font>
       <i val="1"/>
       <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="002F5496"/>
       <sz val="9"/>
     </font>
     <font>
@@ -136,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -162,7 +166,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -171,13 +178,13 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -545,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="135" customWidth="1" min="1" max="1"/>
@@ -607,10 +614,10 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>• The INPUTS box holds business priorities and corporate constraints, with the dates they must be met.</t>
+          <t>• The INPUTS box holds business priorities, corporate constraints, and the data centre / infrastructure overlay, with the dates they must be met.</t>
         </is>
       </c>
     </row>
@@ -631,131 +638,152 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>• All timeline activities are TAM-scoped; BAU roadmap items are excluded. Where an activity directly enables a stated business priority, the cell says so: "[BUILD] … — enabling &lt;priority&gt;".</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>• Tags: [BUILD] = target-state build or adherence · [MIGRATE] = front-book switch, back-book migration or thin-out · [STOP] = stop-sell / stop-integration (frees capacity) · [EXIT] = decommission milestone.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>• Channel / persona context is tagged inline in square brackets where relevant, e.g. [Bank], [ISV], [Wholesale].</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>• Horizons: Now = H2 '26 – H1 '27 · Next = H2 '27 – H1 '29 · Later = H2 '29+.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>• Blue text is a hypothesis to validate. A blank cell means we need your input — not that nothing is planned.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Terminology:</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>• Sales motion = direct, partner-led, or self-serve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>• Persona = the partner or customer type within a segment (e.g. Referral, Agent, ISO/Wholesale, Payfac, PFaaS).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>• Channel = digital, in-person, or omnichannel.</t>
+          <t>• Sales motion = direct, partner-led, or self-serve.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>• Proposition = what the merchant buys (e.g. Genius S, WP360, Revenue Boost). Propositions are inputs and milestones, not an axis of this view.</t>
+          <t>• Persona = the partner or customer type within a segment (e.g. Referral, Agent, ISO/Wholesale, Payfac, PFaaS).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t>• Channel = digital, in-person, or omnichannel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>• Proposition = what the merchant buys (e.g. Genius S, WP360, Revenue Boost). Propositions are inputs and milestones, not an axis of this view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>• Platform = the stack itself, current vs target.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>• Persona treatment: SMB is not split by persona; Integrated is split by persona; Enterprise is to be decided.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>• Persona treatment: SMB is not split by persona; Integrated tags personas inline in brackets; Enterprise is to be decided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Open questions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>1. Which countries do we consider per region? We want to avoid the long tail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>2. Enterprise: do we split by persona / vertical (region × top 1–4 verticals)? Decide before populating.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>3. North America is intentionally omitted from this June pack — it is sequenced for the Jul 20–21 in-person.</t>
+          <t>1. Which countries do we consider per region? We want to avoid the long tail.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>4. Tabs other than UK&amp;I carry pre-fill from the earlier straw man — validate or clear with each geo lead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise notes:</t>
+          <t>2. Enterprise: do we split by persona / vertical (region × top 1–4 verticals)? Decide before populating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>3. Reconcile platform retirement timelines with the data centre consolidation plan — preliminary view requested from infrastructure (an application kept for three years cannot sit in a data centre exiting in one).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>4. North America is intentionally omitted from this June pack — it is sequenced for the Jul 20–21 in-person.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
+          <t>5. Tabs other than UK&amp;I carry pre-fill from the June QPRs and the earlier straw man — validate or clear with each geo lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
           <t>• Persona / vertical split is an open decision. The candidate structure is region × top 1–4 priority verticals (airlines, gambling, QSR/FSR/Stadia…). Decide before populating.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>• Seeded item to validate: WP Total end-of-life — the triPOS option currently points at MBoss, which is not the long-term answer.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>• Seeded item to validate: GMAS EU enterprise back-book → NAP migration as the expansion unlock.</t>
         </is>
@@ -772,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -821,65 +849,77 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Data centre &amp; infrastructure overlay</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Overlay required — application retirement dates must be reconciled with data centre decommissioning timelines (preliminary view requested from infrastructure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING — current stack → target stack → Now / Next / Later</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr"/>
-      <c r="F9" s="12" t="inlineStr"/>
-    </row>
-    <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -896,7 +936,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• API 2.0 / Global API ecosystem on Global Gateway</t>
+            <t>• API 2.0 / Global API on Global Gateway — federated build to the published spec (linting &amp; validation services)</t>
           </r>
           <r>
             <rPr>
@@ -956,18 +996,18 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
-    </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1114,18 +1154,18 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
-    </row>
-    <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr"/>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1142,7 +1182,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• 2/3 analysis in progress — OPEN TAM DECISION</t>
+            <t>• iNASA at launch; target state under 2/3 analysis (decision pending)</t>
           </r>
           <r>
             <rPr>
@@ -1160,7 +1200,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
+            <t>• (to be defined)</t>
           </r>
           <r>
             <rPr>
@@ -1182,18 +1222,18 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
-    </row>
-    <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr"/>
+    </row>
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr"/>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1288,18 +1328,18 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
-    </row>
-    <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr"/>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1316,7 +1356,97 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• Routing 2.0</t>
+            <t>• Routing optimization service — RTR microservice + Prime capabilities extracted from RAFT</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Managed optimization
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Revenue Boost — single orchestration API across credentials, smart retry, fraud and 3DS microservices</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Fraud
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Fraudsight (powered by Ravelin)</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+3DS / exemptions
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• hWP 3DS Flex</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Network tokens / credentials
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• hWP credential management</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Loyalty
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Como</t>
           </r>
           <r>
             <rPr>
@@ -1344,79 +1474,7 @@
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">
-Network tokens
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• hWP tokens</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Loyalty
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Como</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Fraud
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Fraudsight</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Managed optimization
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Revenue Boost</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-FX / DCC / credential mgmt
+FX / DCC
 </t>
           </r>
           <r>
@@ -1426,38 +1484,20 @@
             </rPr>
             <t>• hWP</t>
           </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-3DS / exemptions
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• hWP 3DS flex</t>
-          </r>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-    </row>
-    <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1496,18 +1536,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
-    </row>
-    <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1542,7 +1582,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
+            <t>• (to be defined)</t>
           </r>
           <r>
             <rPr>
@@ -1560,22 +1600,22 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
-    </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+            <t>• (to be defined)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr"/>
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1610,7 +1650,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• WDP</t>
+            <t>• WDP — north star (DMS interim for hGP; Merlin &amp; VAP disputes migrate to WDP in years 1–3; DMS converges to WDP in years 2–5)</t>
           </r>
           <r>
             <rPr>
@@ -1646,21 +1686,22 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• Analysis in progress — OPEN</t>
-          </r>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
+            <t>• Target selection in progress (decision pending)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr"/>
+      <c r="E18" s="15" t="inlineStr"/>
+      <c r="F18" s="15" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A8:F8"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1672,7 +1713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1721,65 +1762,77 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Data centre &amp; infrastructure overlay</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Overlay required — application retirement dates must be reconciled with data centre decommissioning timelines (preliminary view requested from infrastructure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING — current stack → target stack → Now / Next / Later</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr"/>
-      <c r="F9" s="12" t="inlineStr"/>
-    </row>
-    <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1796,7 +1849,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• API 2.0 / Global API ecosystem on Global Gateway</t>
+            <t>• API 2.0 / Global API on Global Gateway — federated build to the published spec (linting &amp; validation services)</t>
           </r>
           <r>
             <rPr>
@@ -1856,18 +1909,18 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
-    </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2014,18 +2067,18 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
-    </row>
-    <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr"/>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2042,7 +2095,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• 2/3 analysis in progress — OPEN TAM DECISION</t>
+            <t>• iNASA at launch; target state under 2/3 analysis (decision pending)</t>
           </r>
           <r>
             <rPr>
@@ -2060,7 +2113,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
+            <t>• (to be defined)</t>
           </r>
           <r>
             <rPr>
@@ -2082,18 +2135,18 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
-    </row>
-    <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr"/>
+    </row>
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr"/>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2188,18 +2241,18 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
-    </row>
-    <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr"/>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2216,7 +2269,97 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• Routing 2.0</t>
+            <t>• Routing optimization service — RTR microservice + Prime capabilities extracted from RAFT</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Managed optimization
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Revenue Boost — single orchestration API across credentials, smart retry, fraud and 3DS microservices</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Fraud
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Fraudsight (powered by Ravelin)</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+3DS / exemptions
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• hWP 3DS Flex</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Network tokens / credentials
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• hWP credential management</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Loyalty
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Como</t>
           </r>
           <r>
             <rPr>
@@ -2244,79 +2387,7 @@
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">
-Network tokens
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• hWP tokens</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Loyalty
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Como</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Fraud
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Fraudsight</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Managed optimization
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Revenue Boost</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-FX / DCC / credential mgmt
+FX / DCC
 </t>
           </r>
           <r>
@@ -2326,38 +2397,20 @@
             </rPr>
             <t>• hWP</t>
           </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-3DS / exemptions
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• hWP 3DS flex</t>
-          </r>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-    </row>
-    <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2396,18 +2449,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
-    </row>
-    <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2442,7 +2495,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
+            <t>• (to be defined)</t>
           </r>
           <r>
             <rPr>
@@ -2460,22 +2513,22 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
-    </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+            <t>• (to be defined)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr"/>
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2510,7 +2563,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• WDP</t>
+            <t>• WDP — north star (DMS interim for hGP; Merlin &amp; VAP disputes migrate to WDP in years 1–3; DMS converges to WDP in years 2–5)</t>
           </r>
           <r>
             <rPr>
@@ -2546,21 +2599,22 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• Analysis in progress — OPEN</t>
-          </r>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
+            <t>• Target selection in progress (decision pending)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr"/>
+      <c r="E18" s="15" t="inlineStr"/>
+      <c r="F18" s="15" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A8:F8"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2572,7 +2626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2621,65 +2675,77 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Data centre &amp; infrastructure overlay</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Overlay required — application retirement dates must be reconciled with data centre decommissioning timelines (preliminary view requested from infrastructure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING — current stack → target stack → Now / Next / Later</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr"/>
-      <c r="F9" s="12" t="inlineStr"/>
-    </row>
-    <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2696,7 +2762,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• API 2.0 / Global API ecosystem on Global Gateway</t>
+            <t>• API 2.0 / Global API on Global Gateway — federated build to the published spec (linting &amp; validation services)</t>
           </r>
           <r>
             <rPr>
@@ -2756,18 +2822,18 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
-    </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2914,18 +2980,18 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
-    </row>
-    <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr"/>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2942,7 +3008,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• 2/3 analysis in progress — OPEN TAM DECISION</t>
+            <t>• iNASA at launch; target state under 2/3 analysis (decision pending)</t>
           </r>
           <r>
             <rPr>
@@ -2960,7 +3026,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
+            <t>• (to be defined)</t>
           </r>
           <r>
             <rPr>
@@ -2982,18 +3048,18 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
-    </row>
-    <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr"/>
+    </row>
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr"/>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3088,18 +3154,18 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
-    </row>
-    <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr"/>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3116,7 +3182,97 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• Routing 2.0</t>
+            <t>• Routing optimization service — RTR microservice + Prime capabilities extracted from RAFT</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Managed optimization
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Revenue Boost — single orchestration API across credentials, smart retry, fraud and 3DS microservices</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Fraud
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Fraudsight (powered by Ravelin)</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+3DS / exemptions
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• hWP 3DS Flex</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Network tokens / credentials
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• hWP credential management</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Loyalty
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Como</t>
           </r>
           <r>
             <rPr>
@@ -3144,79 +3300,7 @@
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">
-Network tokens
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• hWP tokens</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Loyalty
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Como</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Fraud
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Fraudsight</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-Managed optimization
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• Revenue Boost</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-FX / DCC / credential mgmt
+FX / DCC
 </t>
           </r>
           <r>
@@ -3226,38 +3310,20 @@
             </rPr>
             <t>• hWP</t>
           </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">
-3DS / exemptions
-</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="002F5496"/>
-              <sz val="9"/>
-            </rPr>
-            <t>• hWP 3DS flex</t>
-          </r>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-    </row>
-    <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3296,18 +3362,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
-    </row>
-    <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3342,7 +3408,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
+            <t>• (to be defined)</t>
           </r>
           <r>
             <rPr>
@@ -3360,22 +3426,22 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• (open)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
-    </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+            <t>• (to be defined)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr"/>
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3410,7 +3476,7 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• WDP</t>
+            <t>• WDP — north star (DMS interim for hGP; Merlin &amp; VAP disputes migrate to WDP in years 1–3; DMS converges to WDP in years 2–5)</t>
           </r>
           <r>
             <rPr>
@@ -3446,21 +3512,22 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• Analysis in progress — OPEN</t>
-          </r>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
+            <t>• Target selection in progress (decision pending)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr"/>
+      <c r="E18" s="15" t="inlineStr"/>
+      <c r="F18" s="15" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A8:F8"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>